<commit_message>
feat: Restructure UI to Excel-only mode, build dynamic Process Explorer tree, and add persistent IndexedDB file linking
</commit_message>
<xml_diff>
--- a/PM_db.xlsx
+++ b/PM_db.xlsx
@@ -5276,10 +5276,10 @@
         <v>50</v>
       </c>
       <c r="V55">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="W55">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="X55" t="str">
         <v>down</v>
@@ -5365,10 +5365,10 @@
         <v>50</v>
       </c>
       <c r="V56">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="W56">
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="X56" t="str">
         <v>default</v>
@@ -5761,10 +5761,75 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:J2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Account</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Process</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Activity</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Column ID</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Column Name</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Header BG</v>
+      </c>
+      <c r="G1" t="str">
+        <v>BG Color</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Border Color</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Font Color</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Order</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Genpact Solutions</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Direct Procurement</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Port</v>
+      </c>
+      <c r="D2" t="str">
+        <v>lane-1779182539352-m6ugc</v>
+      </c>
+      <c r="E2" t="str">
+        <v>New Lane</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5986,7 +6051,7 @@
         <v>20</v>
       </c>
       <c r="H6" t="str">
-        <v>horizontal</v>
+        <v>grid</v>
       </c>
       <c r="I6">
         <v>80</v>

</xml_diff>

<commit_message>
chore: Clean up sample resources, template JSONs, and sync local Excel database changes
</commit_message>
<xml_diff>
--- a/PM_db.xlsx
+++ b/PM_db.xlsx
@@ -2994,13 +2994,13 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C30" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D30" t="str">
         <v>S1</v>
       </c>
       <c r="E30" t="str">
-        <v>Start</v>
+        <v>Start-cost</v>
       </c>
       <c r="F30" t="str">
         <v>Start</v>
@@ -3009,7 +3009,7 @@
         <v>start</v>
       </c>
       <c r="H30" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779122312233-8jocp</v>
       </c>
       <c r="I30" t="str">
         <v/>
@@ -3051,13 +3051,13 @@
         <v>50</v>
       </c>
       <c r="V30">
-        <v>140</v>
+        <v>72</v>
       </c>
       <c r="W30">
-        <v>512</v>
+        <v>256</v>
       </c>
       <c r="X30" t="str">
-        <v>up</v>
+        <v>default</v>
       </c>
       <c r="Y30" t="str">
         <v>default</v>
@@ -3083,22 +3083,22 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C31" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D31" t="str">
         <v>S2</v>
       </c>
       <c r="E31" t="str">
-        <v>Estimate the safety stock needed based on back orders and inventory on hand for Cisco equipment and prioritize based on install date/lead time</v>
+        <v>Send PO to suppliers</v>
       </c>
       <c r="F31" t="str">
-        <v>Estimate the safety stock needed based on back orders and inventory on hand for Cisco equipment and prioritize based on install date/lead time</v>
+        <v>Send PO to suppliers</v>
       </c>
       <c r="G31" t="str">
         <v>process</v>
       </c>
       <c r="H31" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779122312233-8jocp</v>
       </c>
       <c r="I31" t="str">
         <v/>
@@ -3137,16 +3137,16 @@
         <v>150</v>
       </c>
       <c r="U31">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="V31">
-        <v>125</v>
+        <v>257</v>
       </c>
       <c r="W31">
-        <v>402</v>
+        <v>251</v>
       </c>
       <c r="X31" t="str">
-        <v>up</v>
+        <v>down</v>
       </c>
       <c r="Y31" t="str">
         <v>default</v>
@@ -3172,22 +3172,22 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C32" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D32" t="str">
         <v>S3</v>
       </c>
       <c r="E32" t="str">
-        <v>Update the proposed order quantity in an excel sheet and get it approved by CDK procurement</v>
+        <v>Review price and quantity</v>
       </c>
       <c r="F32" t="str">
-        <v>Update the proposed order quantity in an excel sheet and get it approved by CDK procurement</v>
+        <v>Review price and quantity</v>
       </c>
       <c r="G32" t="str">
         <v>process</v>
       </c>
       <c r="H32" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779122312233-ke65q</v>
       </c>
       <c r="I32" t="str">
         <v/>
@@ -3226,16 +3226,16 @@
         <v>150</v>
       </c>
       <c r="U32">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="V32">
-        <v>125</v>
+        <v>258</v>
       </c>
       <c r="W32">
-        <v>282</v>
+        <v>395</v>
       </c>
       <c r="X32" t="str">
-        <v>up</v>
+        <v>default</v>
       </c>
       <c r="Y32" t="str">
         <v>default</v>
@@ -3261,22 +3261,22 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C33" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D33" t="str">
         <v>S4</v>
       </c>
       <c r="E33" t="str">
-        <v>Approve Safety Stock for Cisco equipment</v>
+        <v>Send the invoice</v>
       </c>
       <c r="F33" t="str">
-        <v>Approve Safety Stock for Cisco equipment</v>
+        <v>Send the invoice</v>
       </c>
       <c r="G33" t="str">
         <v>process</v>
       </c>
       <c r="H33" t="str">
-        <v>lane-1779124199634-jh0dl</v>
+        <v>lane-1779122312233-ke65q</v>
       </c>
       <c r="I33" t="str">
         <v/>
@@ -3315,16 +3315,16 @@
         <v>150</v>
       </c>
       <c r="U33">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="V33">
-        <v>125</v>
+        <v>473</v>
       </c>
       <c r="W33">
-        <v>100</v>
+        <v>394</v>
       </c>
       <c r="X33" t="str">
-        <v>default</v>
+        <v>up</v>
       </c>
       <c r="Y33" t="str">
         <v>default</v>
@@ -3333,7 +3333,7 @@
         <v>default</v>
       </c>
       <c r="AA33" t="str">
-        <v>{"next":{"tgtPort":"top","waypoints":[{"x":386.9049377441406,"y":201.81149291992188}]}}</v>
+        <v>{}</v>
       </c>
       <c r="AB33" t="str">
         <v/>
@@ -3350,34 +3350,34 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C34" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D34" t="str">
         <v>S5</v>
       </c>
       <c r="E34" t="str">
-        <v>E-Mail Cisco to get deal ID</v>
+        <v>Receipted?</v>
       </c>
       <c r="F34" t="str">
-        <v>E-Mail Cisco to get deal ID</v>
+        <v>Receipted?</v>
       </c>
       <c r="G34" t="str">
-        <v>process</v>
+        <v>decision</v>
       </c>
       <c r="H34" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779122312233-8jocp</v>
       </c>
       <c r="I34" t="str">
         <v/>
       </c>
       <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v>S7</v>
+      </c>
+      <c r="L34" t="str">
         <v>S6</v>
-      </c>
-      <c r="K34" t="str">
-        <v/>
-      </c>
-      <c r="L34" t="str">
-        <v/>
       </c>
       <c r="M34" t="str">
         <v>transparent</v>
@@ -3401,25 +3401,25 @@
         <v>No</v>
       </c>
       <c r="T34">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="U34">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="V34">
-        <v>312</v>
+        <v>482</v>
       </c>
       <c r="W34">
-        <v>286</v>
+        <v>232</v>
       </c>
       <c r="X34" t="str">
-        <v>down</v>
+        <v>default</v>
       </c>
       <c r="Y34" t="str">
-        <v>default</v>
+        <v>left</v>
       </c>
       <c r="Z34" t="str">
-        <v>default</v>
+        <v>right</v>
       </c>
       <c r="AA34" t="str">
         <v>{}</v>
@@ -3439,28 +3439,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C35" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D35" t="str">
         <v>S6</v>
       </c>
       <c r="E35" t="str">
-        <v>Provide deal ID – TAT is within the same day (Christine is the contact)</v>
+        <v>Update the PO cost</v>
       </c>
       <c r="F35" t="str">
-        <v>Provide deal ID – TAT is within the same day (Christine is the contact)</v>
+        <v>Update the PO cost</v>
       </c>
       <c r="G35" t="str">
         <v>process</v>
       </c>
       <c r="H35" t="str">
-        <v>lane-1779124199634-n7v9e</v>
+        <v>lane-1779122312233-8jocp</v>
       </c>
       <c r="I35" t="str">
         <v/>
       </c>
       <c r="J35" t="str">
-        <v>S17</v>
+        <v>S8</v>
       </c>
       <c r="K35" t="str">
         <v/>
@@ -3493,13 +3493,13 @@
         <v>150</v>
       </c>
       <c r="U35">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="V35">
-        <v>314</v>
+        <v>721</v>
       </c>
       <c r="W35">
-        <v>668</v>
+        <v>251</v>
       </c>
       <c r="X35" t="str">
         <v>default</v>
@@ -3511,7 +3511,7 @@
         <v>default</v>
       </c>
       <c r="AA35" t="str">
-        <v>{"next":{"tgtPort":"bottom","waypoints":[{"x":579.6392517089844,"y":621.695556640625}]}}</v>
+        <v>{}</v>
       </c>
       <c r="AB35" t="str">
         <v/>
@@ -3528,22 +3528,22 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C36" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D36" t="str">
         <v>S7</v>
       </c>
       <c r="E36" t="str">
-        <v>Log into Cisco CCW portal, go to orders and click create orders</v>
+        <v>Manually update the cost and process the invoice</v>
       </c>
       <c r="F36" t="str">
-        <v>Log into Cisco CCW portal, go to orders and click create orders</v>
+        <v>Manually update the cost and process the invoice</v>
       </c>
       <c r="G36" t="str">
         <v>process</v>
       </c>
       <c r="H36" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779122312233-8jocp</v>
       </c>
       <c r="I36" t="str">
         <v/>
@@ -3558,7 +3558,7 @@
         <v/>
       </c>
       <c r="M36" t="str">
-        <v>transparent</v>
+        <v>#fee1e1</v>
       </c>
       <c r="N36" t="str">
         <v>#000000</v>
@@ -3585,10 +3585,10 @@
         <v>80</v>
       </c>
       <c r="V36">
-        <v>506</v>
+        <v>473</v>
       </c>
       <c r="W36">
-        <v>290</v>
+        <v>100</v>
       </c>
       <c r="X36" t="str">
         <v>default</v>
@@ -3617,28 +3617,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C37" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D37" t="str">
         <v>S8</v>
       </c>
       <c r="E37" t="str">
-        <v>Use the Deal ID to extract the order information</v>
+        <v>End</v>
       </c>
       <c r="F37" t="str">
-        <v>Use the Deal ID to extract the order information</v>
+        <v>End</v>
       </c>
       <c r="G37" t="str">
-        <v>process</v>
+        <v>end</v>
       </c>
       <c r="H37" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779122312233-8jocp</v>
       </c>
       <c r="I37" t="str">
         <v/>
       </c>
       <c r="J37" t="str">
-        <v>S9</v>
+        <v/>
       </c>
       <c r="K37" t="str">
         <v/>
@@ -3668,16 +3668,16 @@
         <v>No</v>
       </c>
       <c r="T37">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="U37">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="V37">
-        <v>716</v>
+        <v>736</v>
       </c>
       <c r="W37">
-        <v>290</v>
+        <v>115</v>
       </c>
       <c r="X37" t="str">
         <v>default</v>
@@ -3706,28 +3706,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C38" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Port</v>
       </c>
       <c r="D38" t="str">
-        <v>S9</v>
+        <v>S1</v>
       </c>
       <c r="E38" t="str">
-        <v>Update details such as Bill to contact, end customer address, end customer contact</v>
+        <v>Start</v>
       </c>
       <c r="F38" t="str">
-        <v>Update details such as Bill to contact, end customer address, end customer contact</v>
+        <v>Start process</v>
       </c>
       <c r="G38" t="str">
-        <v>process</v>
+        <v>start</v>
       </c>
       <c r="H38" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779163665276</v>
       </c>
       <c r="I38" t="str">
         <v/>
       </c>
       <c r="J38" t="str">
-        <v>S10</v>
+        <v>S2</v>
       </c>
       <c r="K38" t="str">
         <v/>
@@ -3757,19 +3757,19 @@
         <v>No</v>
       </c>
       <c r="T38">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="U38">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="V38">
-        <v>929</v>
+        <v>70</v>
       </c>
       <c r="W38">
-        <v>290</v>
+        <v>140</v>
       </c>
       <c r="X38" t="str">
-        <v>default</v>
+        <v>down</v>
       </c>
       <c r="Y38" t="str">
         <v>default</v>
@@ -3795,28 +3795,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C39" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Port</v>
       </c>
       <c r="D39" t="str">
-        <v>S10</v>
+        <v>S2</v>
       </c>
       <c r="E39" t="str">
-        <v>Select items to order</v>
+        <v>End</v>
       </c>
       <c r="F39" t="str">
-        <v>Select items to order</v>
+        <v>End process</v>
       </c>
       <c r="G39" t="str">
-        <v>process</v>
+        <v>end</v>
       </c>
       <c r="H39" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779163665276</v>
       </c>
       <c r="I39" t="str">
         <v/>
       </c>
       <c r="J39" t="str">
-        <v>S11</v>
+        <v/>
       </c>
       <c r="K39" t="str">
         <v/>
@@ -3846,16 +3846,16 @@
         <v>No</v>
       </c>
       <c r="T39">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="U39">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="V39">
-        <v>1136</v>
+        <v>70</v>
       </c>
       <c r="W39">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="X39" t="str">
         <v>default</v>
@@ -3867,7 +3867,7 @@
         <v>default</v>
       </c>
       <c r="AA39" t="str">
-        <v>{"next":{"srcPort":"bottom","tgtPort":"top"}}</v>
+        <v>{}</v>
       </c>
       <c r="AB39" t="str">
         <v/>
@@ -3887,16 +3887,16 @@
         <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D40" t="str">
-        <v>S11</v>
+        <v>S1</v>
       </c>
       <c r="E40" t="str">
-        <v>Split lines to update the order for the required quantity. Repeat the same process for each line item</v>
+        <v>Start</v>
       </c>
       <c r="F40" t="str">
-        <v>Split lines to update the order for the required quantity. Repeat the same process for each line item</v>
+        <v>Start</v>
       </c>
       <c r="G40" t="str">
-        <v>process</v>
+        <v>start</v>
       </c>
       <c r="H40" t="str">
         <v>lane-1779124199634-w7qji</v>
@@ -3905,7 +3905,7 @@
         <v/>
       </c>
       <c r="J40" t="str">
-        <v>S12</v>
+        <v>S2</v>
       </c>
       <c r="K40" t="str">
         <v/>
@@ -3935,19 +3935,19 @@
         <v>No</v>
       </c>
       <c r="T40">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="U40">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="V40">
-        <v>712</v>
+        <v>140</v>
       </c>
       <c r="W40">
-        <v>412</v>
+        <v>546</v>
       </c>
       <c r="X40" t="str">
-        <v>default</v>
+        <v>up</v>
       </c>
       <c r="Y40" t="str">
         <v>default</v>
@@ -3976,13 +3976,13 @@
         <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D41" t="str">
-        <v>S12</v>
+        <v>S2</v>
       </c>
       <c r="E41" t="str">
-        <v>Select the split lines to be ordered and update the purchase order number – Is there a PO created in Oracle?</v>
+        <v>Estimate the safety stock needed based on back orders and inventory on hand for Cisco equipment and prioritize based on install date/lead time</v>
       </c>
       <c r="F41" t="str">
-        <v>Select the split lines to be ordered and update the purchase order number – Is there a PO created in Oracle?</v>
+        <v>Estimate the safety stock needed based on back orders and inventory on hand for Cisco equipment and prioritize based on install date/lead time</v>
       </c>
       <c r="G41" t="str">
         <v>process</v>
@@ -3994,7 +3994,7 @@
         <v/>
       </c>
       <c r="J41" t="str">
-        <v>S13</v>
+        <v>S3</v>
       </c>
       <c r="K41" t="str">
         <v/>
@@ -4027,16 +4027,16 @@
         <v>150</v>
       </c>
       <c r="U41">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="V41">
-        <v>935</v>
+        <v>125</v>
       </c>
       <c r="W41">
-        <v>412</v>
+        <v>402</v>
       </c>
       <c r="X41" t="str">
-        <v>default</v>
+        <v>up</v>
       </c>
       <c r="Y41" t="str">
         <v>default</v>
@@ -4065,13 +4065,13 @@
         <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D42" t="str">
-        <v>S13</v>
+        <v>S3</v>
       </c>
       <c r="E42" t="str">
-        <v>Update other details shipping contact, % discount, request date and save to continue</v>
+        <v>Update the proposed order quantity in an excel sheet and get it approved by CDK procurement</v>
       </c>
       <c r="F42" t="str">
-        <v>Update other details shipping contact, % discount, request date and save to continue</v>
+        <v>Update the proposed order quantity in an excel sheet and get it approved by CDK procurement</v>
       </c>
       <c r="G42" t="str">
         <v>process</v>
@@ -4083,7 +4083,7 @@
         <v/>
       </c>
       <c r="J42" t="str">
-        <v>S14</v>
+        <v>S4</v>
       </c>
       <c r="K42" t="str">
         <v/>
@@ -4116,16 +4116,16 @@
         <v>150</v>
       </c>
       <c r="U42">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="V42">
-        <v>1127</v>
+        <v>125</v>
       </c>
       <c r="W42">
-        <v>412</v>
+        <v>282</v>
       </c>
       <c r="X42" t="str">
-        <v>default</v>
+        <v>up</v>
       </c>
       <c r="Y42" t="str">
         <v>default</v>
@@ -4154,25 +4154,25 @@
         <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D43" t="str">
-        <v>S14</v>
+        <v>S4</v>
       </c>
       <c r="E43" t="str">
-        <v>Set taxability to resale and update special notes</v>
+        <v>Approve Safety Stock for Cisco equipment</v>
       </c>
       <c r="F43" t="str">
-        <v>Set taxability to resale and update special notes</v>
+        <v>Approve Safety Stock for Cisco equipment</v>
       </c>
       <c r="G43" t="str">
         <v>process</v>
       </c>
       <c r="H43" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779124199634-jh0dl</v>
       </c>
       <c r="I43" t="str">
         <v/>
       </c>
       <c r="J43" t="str">
-        <v>S15</v>
+        <v>S5</v>
       </c>
       <c r="K43" t="str">
         <v/>
@@ -4208,10 +4208,10 @@
         <v>80</v>
       </c>
       <c r="V43">
-        <v>1342</v>
+        <v>125</v>
       </c>
       <c r="W43">
-        <v>412</v>
+        <v>100</v>
       </c>
       <c r="X43" t="str">
         <v>default</v>
@@ -4223,7 +4223,7 @@
         <v>default</v>
       </c>
       <c r="AA43" t="str">
-        <v>{}</v>
+        <v>{"next":{"tgtPort":"top","waypoints":[{"x":386.9049377441406,"y":201.81149291992188}]}}</v>
       </c>
       <c r="AB43" t="str">
         <v/>
@@ -4243,13 +4243,13 @@
         <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D44" t="str">
-        <v>S15</v>
+        <v>S5</v>
       </c>
       <c r="E44" t="str">
-        <v>Submit</v>
+        <v>E-Mail Cisco to get deal ID</v>
       </c>
       <c r="F44" t="str">
-        <v>Submit</v>
+        <v>E-Mail Cisco to get deal ID</v>
       </c>
       <c r="G44" t="str">
         <v>process</v>
@@ -4261,7 +4261,7 @@
         <v/>
       </c>
       <c r="J44" t="str">
-        <v>S16</v>
+        <v>S6</v>
       </c>
       <c r="K44" t="str">
         <v/>
@@ -4297,13 +4297,13 @@
         <v>80</v>
       </c>
       <c r="V44">
-        <v>1343</v>
+        <v>312</v>
       </c>
       <c r="W44">
-        <v>526</v>
+        <v>286</v>
       </c>
       <c r="X44" t="str">
-        <v>default</v>
+        <v>down</v>
       </c>
       <c r="Y44" t="str">
         <v>default</v>
@@ -4332,25 +4332,25 @@
         <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D45" t="str">
-        <v>S16</v>
+        <v>S6</v>
       </c>
       <c r="E45" t="str">
-        <v>End</v>
+        <v>Provide deal ID – TAT is within the same day (Christine is the contact)</v>
       </c>
       <c r="F45" t="str">
-        <v>End</v>
+        <v>Provide deal ID – TAT is within the same day (Christine is the contact)</v>
       </c>
       <c r="G45" t="str">
-        <v>end</v>
+        <v>process</v>
       </c>
       <c r="H45" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779124199634-n7v9e</v>
       </c>
       <c r="I45" t="str">
         <v/>
       </c>
       <c r="J45" t="str">
-        <v/>
+        <v>S17</v>
       </c>
       <c r="K45" t="str">
         <v/>
@@ -4380,16 +4380,16 @@
         <v>No</v>
       </c>
       <c r="T45">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="U45">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="V45">
-        <v>1162</v>
+        <v>314</v>
       </c>
       <c r="W45">
-        <v>541</v>
+        <v>668</v>
       </c>
       <c r="X45" t="str">
         <v>default</v>
@@ -4401,7 +4401,7 @@
         <v>default</v>
       </c>
       <c r="AA45" t="str">
-        <v>{}</v>
+        <v>{"next":{"tgtPort":"bottom","waypoints":[{"x":579.6392517089844,"y":621.695556640625}]}}</v>
       </c>
       <c r="AB45" t="str">
         <v/>
@@ -4421,13 +4421,13 @@
         <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D46" t="str">
-        <v>S17</v>
+        <v>S7</v>
       </c>
       <c r="E46" t="str">
-        <v>Create Manual PO in Oracle EBS and get it Approved</v>
+        <v>Log into Cisco CCW portal, go to orders and click create orders</v>
       </c>
       <c r="F46" t="str">
-        <v/>
+        <v>Log into Cisco CCW portal, go to orders and click create orders</v>
       </c>
       <c r="G46" t="str">
         <v>process</v>
@@ -4439,7 +4439,7 @@
         <v/>
       </c>
       <c r="J46" t="str">
-        <v>S7</v>
+        <v>S8</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -4472,13 +4472,13 @@
         <v>150</v>
       </c>
       <c r="U46">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="V46">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="W46">
-        <v>529</v>
+        <v>290</v>
       </c>
       <c r="X46" t="str">
         <v>default</v>
@@ -4507,28 +4507,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C47" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D47" t="str">
-        <v>S1</v>
+        <v>S8</v>
       </c>
       <c r="E47" t="str">
-        <v>Start-cost</v>
+        <v>Use the Deal ID to extract the order information</v>
       </c>
       <c r="F47" t="str">
-        <v>Start</v>
+        <v>Use the Deal ID to extract the order information</v>
       </c>
       <c r="G47" t="str">
-        <v>start</v>
+        <v>process</v>
       </c>
       <c r="H47" t="str">
-        <v>lane-1779122312233-8jocp</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I47" t="str">
         <v/>
       </c>
       <c r="J47" t="str">
-        <v>S2</v>
+        <v>S9</v>
       </c>
       <c r="K47" t="str">
         <v/>
@@ -4558,16 +4558,16 @@
         <v>No</v>
       </c>
       <c r="T47">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="U47">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="V47">
-        <v>72</v>
+        <v>716</v>
       </c>
       <c r="W47">
-        <v>256</v>
+        <v>290</v>
       </c>
       <c r="X47" t="str">
         <v>default</v>
@@ -4596,28 +4596,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C48" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D48" t="str">
-        <v>S2</v>
+        <v>S9</v>
       </c>
       <c r="E48" t="str">
-        <v>Send PO to suppliers</v>
+        <v>Update details such as Bill to contact, end customer address, end customer contact</v>
       </c>
       <c r="F48" t="str">
-        <v>Send PO to suppliers</v>
+        <v>Update details such as Bill to contact, end customer address, end customer contact</v>
       </c>
       <c r="G48" t="str">
         <v>process</v>
       </c>
       <c r="H48" t="str">
-        <v>lane-1779122312233-8jocp</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I48" t="str">
         <v/>
       </c>
       <c r="J48" t="str">
-        <v>S3</v>
+        <v>S10</v>
       </c>
       <c r="K48" t="str">
         <v/>
@@ -4650,16 +4650,16 @@
         <v>150</v>
       </c>
       <c r="U48">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="V48">
-        <v>257</v>
+        <v>929</v>
       </c>
       <c r="W48">
-        <v>251</v>
+        <v>290</v>
       </c>
       <c r="X48" t="str">
-        <v>down</v>
+        <v>default</v>
       </c>
       <c r="Y48" t="str">
         <v>default</v>
@@ -4685,28 +4685,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C49" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D49" t="str">
-        <v>S3</v>
+        <v>S10</v>
       </c>
       <c r="E49" t="str">
-        <v>Review price and quantity</v>
+        <v>Select items to order</v>
       </c>
       <c r="F49" t="str">
-        <v>Review price and quantity</v>
+        <v>Select items to order</v>
       </c>
       <c r="G49" t="str">
         <v>process</v>
       </c>
       <c r="H49" t="str">
-        <v>lane-1779122312233-ke65q</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I49" t="str">
         <v/>
       </c>
       <c r="J49" t="str">
-        <v>S4</v>
+        <v>S11</v>
       </c>
       <c r="K49" t="str">
         <v/>
@@ -4739,13 +4739,13 @@
         <v>150</v>
       </c>
       <c r="U49">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="V49">
-        <v>258</v>
+        <v>1136</v>
       </c>
       <c r="W49">
-        <v>395</v>
+        <v>290</v>
       </c>
       <c r="X49" t="str">
         <v>default</v>
@@ -4757,7 +4757,7 @@
         <v>default</v>
       </c>
       <c r="AA49" t="str">
-        <v>{}</v>
+        <v>{"next":{"srcPort":"bottom","tgtPort":"top"}}</v>
       </c>
       <c r="AB49" t="str">
         <v/>
@@ -4774,28 +4774,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C50" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D50" t="str">
-        <v>S4</v>
+        <v>S11</v>
       </c>
       <c r="E50" t="str">
-        <v>Send the invoice</v>
+        <v>Split lines to update the order for the required quantity. Repeat the same process for each line item</v>
       </c>
       <c r="F50" t="str">
-        <v>Send the invoice</v>
+        <v>Split lines to update the order for the required quantity. Repeat the same process for each line item</v>
       </c>
       <c r="G50" t="str">
         <v>process</v>
       </c>
       <c r="H50" t="str">
-        <v>lane-1779122312233-ke65q</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I50" t="str">
         <v/>
       </c>
       <c r="J50" t="str">
-        <v>S5</v>
+        <v>S12</v>
       </c>
       <c r="K50" t="str">
         <v/>
@@ -4828,16 +4828,16 @@
         <v>150</v>
       </c>
       <c r="U50">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="V50">
-        <v>473</v>
+        <v>712</v>
       </c>
       <c r="W50">
-        <v>394</v>
+        <v>412</v>
       </c>
       <c r="X50" t="str">
-        <v>up</v>
+        <v>default</v>
       </c>
       <c r="Y50" t="str">
         <v>default</v>
@@ -4863,34 +4863,34 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C51" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D51" t="str">
-        <v>S5</v>
+        <v>S12</v>
       </c>
       <c r="E51" t="str">
-        <v>Receipted?</v>
+        <v>Select the split lines to be ordered and update the purchase order number – Is there a PO created in Oracle?</v>
       </c>
       <c r="F51" t="str">
-        <v>Receipted?</v>
+        <v>Select the split lines to be ordered and update the purchase order number – Is there a PO created in Oracle?</v>
       </c>
       <c r="G51" t="str">
-        <v>decision</v>
+        <v>process</v>
       </c>
       <c r="H51" t="str">
-        <v>lane-1779122312233-8jocp</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I51" t="str">
         <v/>
       </c>
       <c r="J51" t="str">
-        <v/>
+        <v>S13</v>
       </c>
       <c r="K51" t="str">
-        <v>S7</v>
+        <v/>
       </c>
       <c r="L51" t="str">
-        <v>S6</v>
+        <v/>
       </c>
       <c r="M51" t="str">
         <v>transparent</v>
@@ -4914,25 +4914,25 @@
         <v>No</v>
       </c>
       <c r="T51">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="U51">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="V51">
-        <v>482</v>
+        <v>935</v>
       </c>
       <c r="W51">
-        <v>232</v>
+        <v>412</v>
       </c>
       <c r="X51" t="str">
         <v>default</v>
       </c>
       <c r="Y51" t="str">
-        <v>left</v>
+        <v>default</v>
       </c>
       <c r="Z51" t="str">
-        <v>right</v>
+        <v>default</v>
       </c>
       <c r="AA51" t="str">
         <v>{}</v>
@@ -4952,28 +4952,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C52" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D52" t="str">
-        <v>S6</v>
+        <v>S13</v>
       </c>
       <c r="E52" t="str">
-        <v>Update the PO cost</v>
+        <v>Update other details shipping contact, % discount, request date and save to continue</v>
       </c>
       <c r="F52" t="str">
-        <v>Update the PO cost</v>
+        <v>Update other details shipping contact, % discount, request date and save to continue</v>
       </c>
       <c r="G52" t="str">
         <v>process</v>
       </c>
       <c r="H52" t="str">
-        <v>lane-1779122312233-8jocp</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I52" t="str">
         <v/>
       </c>
       <c r="J52" t="str">
-        <v>S8</v>
+        <v>S14</v>
       </c>
       <c r="K52" t="str">
         <v/>
@@ -5006,13 +5006,13 @@
         <v>150</v>
       </c>
       <c r="U52">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="V52">
-        <v>721</v>
+        <v>1127</v>
       </c>
       <c r="W52">
-        <v>251</v>
+        <v>412</v>
       </c>
       <c r="X52" t="str">
         <v>default</v>
@@ -5041,28 +5041,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C53" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D53" t="str">
-        <v>S7</v>
+        <v>S14</v>
       </c>
       <c r="E53" t="str">
-        <v>Manually update the cost and process the invoice</v>
+        <v>Set taxability to resale and update special notes</v>
       </c>
       <c r="F53" t="str">
-        <v>Manually update the cost and process the invoice</v>
+        <v>Set taxability to resale and update special notes</v>
       </c>
       <c r="G53" t="str">
         <v>process</v>
       </c>
       <c r="H53" t="str">
-        <v>lane-1779122312233-8jocp</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I53" t="str">
         <v/>
       </c>
       <c r="J53" t="str">
-        <v>S8</v>
+        <v>S15</v>
       </c>
       <c r="K53" t="str">
         <v/>
@@ -5071,7 +5071,7 @@
         <v/>
       </c>
       <c r="M53" t="str">
-        <v>#fee1e1</v>
+        <v>transparent</v>
       </c>
       <c r="N53" t="str">
         <v>#000000</v>
@@ -5098,10 +5098,10 @@
         <v>80</v>
       </c>
       <c r="V53">
-        <v>473</v>
+        <v>1342</v>
       </c>
       <c r="W53">
-        <v>100</v>
+        <v>412</v>
       </c>
       <c r="X53" t="str">
         <v>default</v>
@@ -5130,28 +5130,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C54" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D54" t="str">
-        <v>S8</v>
+        <v>S15</v>
       </c>
       <c r="E54" t="str">
-        <v>End</v>
+        <v>Submit</v>
       </c>
       <c r="F54" t="str">
-        <v>End</v>
+        <v>Submit</v>
       </c>
       <c r="G54" t="str">
-        <v>end</v>
+        <v>process</v>
       </c>
       <c r="H54" t="str">
-        <v>lane-1779122312233-8jocp</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I54" t="str">
         <v/>
       </c>
       <c r="J54" t="str">
-        <v/>
+        <v>S16</v>
       </c>
       <c r="K54" t="str">
         <v/>
@@ -5181,16 +5181,16 @@
         <v>No</v>
       </c>
       <c r="T54">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="U54">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="V54">
-        <v>736</v>
+        <v>1343</v>
       </c>
       <c r="W54">
-        <v>115</v>
+        <v>526</v>
       </c>
       <c r="X54" t="str">
         <v>default</v>
@@ -5219,28 +5219,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C55" t="str">
-        <v>Port</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D55" t="str">
-        <v>S1</v>
+        <v>S16</v>
       </c>
       <c r="E55" t="str">
-        <v>Start</v>
+        <v>End</v>
       </c>
       <c r="F55" t="str">
-        <v>Start process</v>
+        <v>End</v>
       </c>
       <c r="G55" t="str">
-        <v>start</v>
+        <v>end</v>
       </c>
       <c r="H55" t="str">
-        <v>lane-1779163665276</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I55" t="str">
         <v/>
       </c>
       <c r="J55" t="str">
-        <v>S2</v>
+        <v/>
       </c>
       <c r="K55" t="str">
         <v/>
@@ -5276,13 +5276,13 @@
         <v>50</v>
       </c>
       <c r="V55">
-        <v>70</v>
+        <v>1162</v>
       </c>
       <c r="W55">
-        <v>140</v>
+        <v>541</v>
       </c>
       <c r="X55" t="str">
-        <v>down</v>
+        <v>default</v>
       </c>
       <c r="Y55" t="str">
         <v>default</v>
@@ -5308,28 +5308,28 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C56" t="str">
-        <v>Port</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D56" t="str">
-        <v>S2</v>
+        <v>S17</v>
       </c>
       <c r="E56" t="str">
-        <v>End</v>
+        <v>Create Manual PO in Oracle EBS and get it Approved</v>
       </c>
       <c r="F56" t="str">
-        <v>End process</v>
+        <v/>
       </c>
       <c r="G56" t="str">
-        <v>end</v>
+        <v>process</v>
       </c>
       <c r="H56" t="str">
-        <v>lane-1779163665276</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="I56" t="str">
         <v/>
       </c>
       <c r="J56" t="str">
-        <v/>
+        <v>S7</v>
       </c>
       <c r="K56" t="str">
         <v/>
@@ -5359,16 +5359,16 @@
         <v>No</v>
       </c>
       <c r="T56">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="U56">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="V56">
-        <v>70</v>
+        <v>505</v>
       </c>
       <c r="W56">
-        <v>270</v>
+        <v>529</v>
       </c>
       <c r="X56" t="str">
         <v>default</v>
@@ -5568,19 +5568,19 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C6" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D6" t="str">
-        <v>lane-1779124199634-w7qji</v>
+        <v>lane-1779122312233-8jocp</v>
       </c>
       <c r="E6" t="str">
-        <v>Direct Procurement Buyers</v>
+        <v>Genpact Direct Procurement Buyers</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>transparent</v>
       </c>
       <c r="G6" t="str">
-        <v/>
+        <v>transparent</v>
       </c>
       <c r="H6" t="str">
         <v>#000000</v>
@@ -5589,7 +5589,7 @@
         <v>#000000</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -5600,13 +5600,13 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C7" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D7" t="str">
-        <v>lane-1779124199634-jh0dl</v>
+        <v>lane-1779122312233-ke65q</v>
       </c>
       <c r="E7" t="str">
-        <v>CDK Procurement</v>
+        <v>Suppliers</v>
       </c>
       <c r="F7" t="str">
         <v>transparent</v>
@@ -5621,7 +5621,7 @@
         <v>#000000</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -5632,13 +5632,13 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C8" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Port</v>
       </c>
       <c r="D8" t="str">
-        <v>lane-1779124199634-n7v9e</v>
+        <v>lane-1779163665276</v>
       </c>
       <c r="E8" t="str">
-        <v>Cisco</v>
+        <v>Department Swimlane 1</v>
       </c>
       <c r="F8" t="str">
         <v>transparent</v>
@@ -5653,7 +5653,7 @@
         <v>#000000</v>
       </c>
       <c r="J8">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -5664,13 +5664,13 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C9" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D9" t="str">
-        <v>lane-1779122312233-8jocp</v>
+        <v>lane-1779124199634-jh0dl</v>
       </c>
       <c r="E9" t="str">
-        <v>Genpact Direct Procurement Buyers</v>
+        <v>CDK Procurement</v>
       </c>
       <c r="F9" t="str">
         <v>transparent</v>
@@ -5696,19 +5696,19 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C10" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D10" t="str">
-        <v>lane-1779122312233-ke65q</v>
+        <v>lane-1779124199634-w7qji</v>
       </c>
       <c r="E10" t="str">
-        <v>Suppliers</v>
+        <v>Direct Procurement Buyers</v>
       </c>
       <c r="F10" t="str">
-        <v>transparent</v>
+        <v/>
       </c>
       <c r="G10" t="str">
-        <v>transparent</v>
+        <v/>
       </c>
       <c r="H10" t="str">
         <v>#000000</v>
@@ -5728,13 +5728,13 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C11" t="str">
-        <v>Port</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D11" t="str">
-        <v>lane-1779163665276</v>
+        <v>lane-1779124199634-n7v9e</v>
       </c>
       <c r="E11" t="str">
-        <v>Department Swimlane 1</v>
+        <v>Cisco</v>
       </c>
       <c r="F11" t="str">
         <v>transparent</v>
@@ -5749,7 +5749,7 @@
         <v>#000000</v>
       </c>
       <c r="J11">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5960,7 +5960,7 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C4" t="str">
-        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
+        <v>Process Direct Procurement Change Order for cost Change</v>
       </c>
       <c r="D4" t="str">
         <v>light</v>
@@ -5998,7 +5998,7 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C5" t="str">
-        <v>Process Direct Procurement Change Order for cost Change</v>
+        <v>Port</v>
       </c>
       <c r="D5" t="str">
         <v>light</v>
@@ -6013,10 +6013,10 @@
         <v>20</v>
       </c>
       <c r="H5" t="str">
-        <v>horizontal</v>
+        <v>grid</v>
       </c>
       <c r="I5">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="J5" t="str">
         <v>horizontal</v>
@@ -6036,7 +6036,7 @@
         <v>Direct Procurement</v>
       </c>
       <c r="C6" t="str">
-        <v>Port</v>
+        <v>Direct Procurement  - Cisco/Meraki Order Processing process (In CCW)</v>
       </c>
       <c r="D6" t="str">
         <v>light</v>
@@ -6051,10 +6051,10 @@
         <v>20</v>
       </c>
       <c r="H6" t="str">
-        <v>grid</v>
+        <v>horizontal</v>
       </c>
       <c r="I6">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="J6" t="str">
         <v>horizontal</v>

</xml_diff>